<commit_message>
feat: Add S beam extractor and S_Beam sheet output
PDF2 p.2 (S大梁リスト) extraction via the same anchor-text approach:
finds SG/CSG anchors, picks up section type (SH-/BH-/H- with 4 dimensions),
connected spans (preserves reading order across continuation rows), and
通り起点/終点 gridline labels.

Excel writer now emits S_Beam sheet alongside RC_Beam, completing the
sample workbook for PDF2 (20 RC beams + 16 S beams). Span numbers are
parsed with thousand-separator awareness ('8,400,7,800' -> [8400, 7800]).
</commit_message>
<xml_diff>
--- a/pdf-to-excel/src/sample-output.xlsx
+++ b/pdf-to-excel/src/sample-output.xlsx
@@ -5,9 +5,9 @@
   <sheets>
     <sheet name="Meta" sheetId="1" r:id="rId1"/>
     <sheet name="RC_Beam" sheetId="2" r:id="rId2"/>
-    <sheet name="RC_Column" sheetId="3" r:id="rId3"/>
-    <sheet name="CFT_Column" sheetId="4" r:id="rId4"/>
-    <sheet name="S_Beam" sheetId="5" r:id="rId5"/>
+    <sheet name="S_Beam" sheetId="3" r:id="rId3"/>
+    <sheet name="RC_Column" sheetId="4" r:id="rId4"/>
+    <sheet name="CFT_Column" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -424,7 +424,7 @@
         <v>source_pdf_filename</v>
       </c>
       <c r="B3" t="str">
-        <v>PDF2-p1-RC基礎大梁.pdf</v>
+        <v>PDF2.pdf</v>
       </c>
     </row>
     <row r="4">
@@ -440,7 +440,7 @@
         <v>drawing_name</v>
       </c>
       <c r="B5" t="str">
-        <v>RC基礎大梁リスト</v>
+        <v>RC基礎大梁リスト + S大梁リスト</v>
       </c>
     </row>
     <row r="6">
@@ -448,7 +448,7 @@
         <v>extracted_at</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-05-20T03:51:48.400Z</v>
+        <v>2026-05-20T04:04:08.081Z</v>
       </c>
     </row>
     <row r="7">
@@ -4112,16 +4112,759 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:N17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>placeholder</v>
+        <v>TypeName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>符号</v>
+      </c>
+      <c r="C1" t="str">
+        <v>断面形式</v>
+      </c>
+      <c r="D1" t="str">
+        <v>成H_mm</v>
+      </c>
+      <c r="E1" t="str">
+        <v>幅B_mm</v>
+      </c>
+      <c r="F1" t="str">
+        <v>ウェブtw_mm</v>
+      </c>
+      <c r="G1" t="str">
+        <v>フランジtf_mm</v>
+      </c>
+      <c r="H1" t="str">
+        <v>スパン_mm</v>
+      </c>
+      <c r="I1" t="str">
+        <v>通り起点</v>
+      </c>
+      <c r="J1" t="str">
+        <v>通り終点</v>
+      </c>
+      <c r="K1" t="str">
+        <v>鋼材グレード</v>
+      </c>
+      <c r="L1" t="str">
+        <v>区分</v>
+      </c>
+      <c r="M1" t="str">
+        <v>原文</v>
+      </c>
+      <c r="N1" t="str">
+        <v>備考</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>SG1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>SG1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D2">
+        <v>600</v>
+      </c>
+      <c r="E2">
+        <v>200</v>
+      </c>
+      <c r="F2">
+        <v>12</v>
+      </c>
+      <c r="G2">
+        <v>16</v>
+      </c>
+      <c r="H2" t="str">
+        <v>8400;7800;6450;6000</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v>SH-600×200×12×16</v>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SG1A</v>
+      </c>
+      <c r="B3" t="str">
+        <v>SG1A</v>
+      </c>
+      <c r="C3" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D3">
+        <v>600</v>
+      </c>
+      <c r="E3">
+        <v>250</v>
+      </c>
+      <c r="F3">
+        <v>12</v>
+      </c>
+      <c r="G3">
+        <v>28</v>
+      </c>
+      <c r="H3" t="str">
+        <v>6450</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Xd1</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Xd2</v>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v>SH-600×250×12×28</v>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>SG2</v>
+      </c>
+      <c r="B4" t="str">
+        <v>SG2</v>
+      </c>
+      <c r="C4" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D4">
+        <v>600</v>
+      </c>
+      <c r="E4">
+        <v>200</v>
+      </c>
+      <c r="F4">
+        <v>12</v>
+      </c>
+      <c r="G4">
+        <v>16</v>
+      </c>
+      <c r="H4" t="str">
+        <v>7800;6450;6000</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Xd1</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Xd9</v>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v>SH-600×200×12×16</v>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>SG2A</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SG2A</v>
+      </c>
+      <c r="C5" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D5">
+        <v>600</v>
+      </c>
+      <c r="E5">
+        <v>250</v>
+      </c>
+      <c r="F5">
+        <v>12</v>
+      </c>
+      <c r="G5">
+        <v>28</v>
+      </c>
+      <c r="H5" t="str">
+        <v>6450</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Xd1</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Xd2</v>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v>SH-600×250×12×28</v>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>SG3</v>
+      </c>
+      <c r="B6" t="str">
+        <v>SG3</v>
+      </c>
+      <c r="C6" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D6">
+        <v>600</v>
+      </c>
+      <c r="E6">
+        <v>200</v>
+      </c>
+      <c r="F6">
+        <v>12</v>
+      </c>
+      <c r="G6">
+        <v>16</v>
+      </c>
+      <c r="H6" t="str">
+        <v>8400;7800</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Xd5</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Xd11</v>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v>SH-600×200×12×16</v>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>SG4</v>
+      </c>
+      <c r="B7" t="str">
+        <v>SG4</v>
+      </c>
+      <c r="C7" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D7">
+        <v>600</v>
+      </c>
+      <c r="E7">
+        <v>250</v>
+      </c>
+      <c r="F7">
+        <v>12</v>
+      </c>
+      <c r="G7">
+        <v>25</v>
+      </c>
+      <c r="H7" t="str">
+        <v>6000</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Xd11</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Xd12</v>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v>SH-600×250×12×25</v>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>SG5</v>
+      </c>
+      <c r="B8" t="str">
+        <v>SG5</v>
+      </c>
+      <c r="C8" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D8">
+        <v>600</v>
+      </c>
+      <c r="E8">
+        <v>250</v>
+      </c>
+      <c r="F8">
+        <v>12</v>
+      </c>
+      <c r="G8">
+        <v>28</v>
+      </c>
+      <c r="H8" t="str">
+        <v>6450</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Xd2</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Xd3</v>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v>SH-600×250×12×28</v>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>SG6</v>
+      </c>
+      <c r="B9" t="str">
+        <v>SG6</v>
+      </c>
+      <c r="C9" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D9">
+        <v>600</v>
+      </c>
+      <c r="E9">
+        <v>300</v>
+      </c>
+      <c r="F9">
+        <v>16</v>
+      </c>
+      <c r="G9">
+        <v>32</v>
+      </c>
+      <c r="H9" t="str">
+        <v>6450</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Xd3</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Xd4</v>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v>SH-600×300×16×32</v>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>SG7</v>
+      </c>
+      <c r="B10" t="str">
+        <v>SG7</v>
+      </c>
+      <c r="C10" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D10">
+        <v>600</v>
+      </c>
+      <c r="E10">
+        <v>250</v>
+      </c>
+      <c r="F10">
+        <v>12</v>
+      </c>
+      <c r="G10">
+        <v>28</v>
+      </c>
+      <c r="H10" t="str">
+        <v>7800</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Xd4</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Xd5</v>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v>SH-600×250×12×28</v>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>SG8</v>
+      </c>
+      <c r="B11" t="str">
+        <v>SG8</v>
+      </c>
+      <c r="C11" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D11">
+        <v>800</v>
+      </c>
+      <c r="E11">
+        <v>400</v>
+      </c>
+      <c r="F11">
+        <v>19</v>
+      </c>
+      <c r="G11">
+        <v>36</v>
+      </c>
+      <c r="H11" t="str">
+        <v>14400;8400</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Xd9</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Xd12</v>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v>SH-800×400×19×36</v>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>SG9</v>
+      </c>
+      <c r="B12" t="str">
+        <v>SG9</v>
+      </c>
+      <c r="C12" t="str">
+        <v>BH</v>
+      </c>
+      <c r="D12">
+        <v>800</v>
+      </c>
+      <c r="E12">
+        <v>400</v>
+      </c>
+      <c r="F12">
+        <v>16</v>
+      </c>
+      <c r="G12">
+        <v>32</v>
+      </c>
+      <c r="H12" t="str">
+        <v>3450</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Xd12</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Xd13</v>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v>BH-800×400×16×32</v>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>SG10</v>
+      </c>
+      <c r="B13" t="str">
+        <v>SG10</v>
+      </c>
+      <c r="C13" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D13">
+        <v>600</v>
+      </c>
+      <c r="E13">
+        <v>300</v>
+      </c>
+      <c r="F13">
+        <v>12</v>
+      </c>
+      <c r="G13">
+        <v>28</v>
+      </c>
+      <c r="H13" t="str">
+        <v>7800;6450</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Xd2</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Xd5</v>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v>SH-600×300×12×28</v>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>SG11</v>
+      </c>
+      <c r="B14" t="str">
+        <v>SG11</v>
+      </c>
+      <c r="C14" t="str">
+        <v>BH</v>
+      </c>
+      <c r="D14">
+        <v>600</v>
+      </c>
+      <c r="E14">
+        <v>350</v>
+      </c>
+      <c r="F14">
+        <v>16</v>
+      </c>
+      <c r="G14">
+        <v>36</v>
+      </c>
+      <c r="H14" t="str">
+        <v>6450</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Xd3</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Xd4</v>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v>BH-600×350×16×36</v>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>CSG3</v>
+      </c>
+      <c r="B15" t="str">
+        <v>CSG3</v>
+      </c>
+      <c r="C15" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D15">
+        <v>800</v>
+      </c>
+      <c r="E15">
+        <v>250</v>
+      </c>
+      <c r="F15">
+        <v>14</v>
+      </c>
+      <c r="G15">
+        <v>22</v>
+      </c>
+      <c r="H15" t="str">
+        <v>3450</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v>SH-800×250×14×22</v>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>CSG5</v>
+      </c>
+      <c r="B16" t="str">
+        <v>CSG5</v>
+      </c>
+      <c r="C16" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D16">
+        <v>600</v>
+      </c>
+      <c r="E16">
+        <v>250</v>
+      </c>
+      <c r="F16">
+        <v>12</v>
+      </c>
+      <c r="G16">
+        <v>25</v>
+      </c>
+      <c r="H16" t="str">
+        <v>1650</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v>SH-600×250×12×25</v>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>CSG6</v>
+      </c>
+      <c r="B17" t="str">
+        <v>CSG6</v>
+      </c>
+      <c r="C17" t="str">
+        <v>SH</v>
+      </c>
+      <c r="D17">
+        <v>600</v>
+      </c>
+      <c r="E17">
+        <v>300</v>
+      </c>
+      <c r="F17">
+        <v>16</v>
+      </c>
+      <c r="G17">
+        <v>32</v>
+      </c>
+      <c r="H17" t="str">
+        <v>4100</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v>SH-600×300×16×32</v>
+      </c>
+      <c r="N17" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: OCR-based column extractor for glyph-obfuscated PDFs
PDF1 (柱リスト) embeds a subsetted MS-UIGothic with the ToUnicode CMap
stripped, so all parsers (pdfjs, poppler, mupdf, ghostscript) return the
same garbled CIDs. Confirmed via probe-font.mjs subagent investigation.

Workaround: render the page to PNG via pdftoppm at 300 DPI, run tesseract
with --psm 11 (sparse text) and -l jpn, then parse the TSV bboxes through
the same anchor pattern used for native text. PSM 11 detects all six
SC anchors cleanly; PSM 6 (block) was missing most of them.

Extractor recognizes SC/CC/CFT/C anchor prefixes and harvests section
strings (□-700x700x25, SH-700x350x16x25 form) from the rectangular area
under each anchor. detectCategory() gets SC/CC/CFT entries so the sheet
is named 柱.

Sample output: 5 of 6 SC columns extracted with their section variants
(SC1, SC2 each have 4 floor-range sections; SC5 has 3). Marked as
"OCR抽出 (低精度)" in the 備考 column.
</commit_message>
<xml_diff>
--- a/pdf-to-excel/src/sample-output.xlsx
+++ b/pdf-to-excel/src/sample-output.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Meta" sheetId="1" r:id="rId1"/>
     <sheet name="基礎大梁" sheetId="2" r:id="rId2"/>
     <sheet name="S大梁" sheetId="3" r:id="rId3"/>
+    <sheet name="柱" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -430,7 +431,7 @@
         <v>extracted_at</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-05-20T04:28:52.877Z</v>
+        <v>2026-05-20T04:34:18.220Z</v>
       </c>
     </row>
     <row r="5">
@@ -446,7 +447,7 @@
         <v>detected_categories</v>
       </c>
       <c r="B6" t="str">
-        <v>RC基礎大梁 (20行), S大梁 (16行)</v>
+        <v>RC基礎大梁 (20行), S大梁 (16行), S柱 (6行) ※OCR</v>
       </c>
     </row>
   </sheetData>
@@ -4178,4 +4179,216 @@
     <ignoredError numberStoredAsText="1" sqref="A1:N18"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G8"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="30.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" t="str">
+        <v>TypeName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>符号</v>
+      </c>
+      <c r="C1" t="str">
+        <v>断面</v>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v>鋼材グレード</v>
+      </c>
+      <c r="F1" t="str">
+        <v>原文</v>
+      </c>
+      <c r="G1" t="str">
+        <v>備考</v>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>断面リスト</v>
+      </c>
+      <c r="D2" t="str">
+        <v>区分数</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SC1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>SC1</v>
+      </c>
+      <c r="C3" t="str">
+        <v>-700x700x25;-700x700x28;-750x750x28;-800x800x28</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>-700x700x25 / -700x700x28 / -750x750x28 / -800x800x28</v>
+      </c>
+      <c r="G3" t="str">
+        <v>OCR抽出 (低精度) — 元PDFがグリフ難読化のためOCRフォールバック</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>SC2</v>
+      </c>
+      <c r="B4" t="str">
+        <v>SC2</v>
+      </c>
+      <c r="C4" t="str">
+        <v>-700x700x25;-700x700x28;-750x750x28;-800x800x28</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v>-700x700x25 / -700x700x28 / -750x750x28 / -800x800x28</v>
+      </c>
+      <c r="G4" t="str">
+        <v>OCR抽出 (低精度) — 元PDFがグリフ難読化のためOCRフォールバック</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>SC3</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SC3</v>
+      </c>
+      <c r="C5" t="str">
+        <v>-450x450x28</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>-450x450x28</v>
+      </c>
+      <c r="G5" t="str">
+        <v>OCR抽出 (低精度) — 元PDFがグリフ難読化のためOCRフォールバック</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>SC4</v>
+      </c>
+      <c r="B6" t="str">
+        <v>SC4</v>
+      </c>
+      <c r="C6" t="str">
+        <v>-400x400x22</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>-400x400x22</v>
+      </c>
+      <c r="G6" t="str">
+        <v>OCR抽出 (低精度) — 元PDFがグリフ難読化のためOCRフォールバック</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>SC5</v>
+      </c>
+      <c r="B7" t="str">
+        <v>SC5</v>
+      </c>
+      <c r="C7" t="str">
+        <v>SH-700x350x16x25;SH-700x350x16x28;SH-700x350x16x36</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>SH-700x350x16x25 / SH-700x350x16x28 / SH-700x350x16x36</v>
+      </c>
+      <c r="G7" t="str">
+        <v>OCR抽出 (低精度) — 元PDFがグリフ難読化のためOCRフォールバック</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>SC6</v>
+      </c>
+      <c r="B8" t="str">
+        <v>SC6</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>OCR抽出 (低精度) — 元PDFがグリフ難読化のためOCRフォールバック</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+  </mergeCells>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>